<commit_message>
manifest and test plan change
</commit_message>
<xml_diff>
--- a/docs/cockpit-zfs-encryption-test-plan.xlsx
+++ b/docs/cockpit-zfs-encryption-test-plan.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="467">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="301">
   <si>
     <t xml:space="preserve">Field</t>
   </si>
@@ -279,117 +279,6 @@
   </si>
   <si>
     <t xml:space="preserve">The snapshot row shows the correct lock icon matching its keystatus (locked/unlocked).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create FS - Passphrase Encryption</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Encryption toggle enables encryption fields</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Navigate to Datasets tab.
-2. Click 'Create File System'.
-3. Select a parent filesystem.
-4. Enter a name.
-5. Toggle 'Encryption' ON.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Encryption is enabled. Passphrase and Confirm Passphrase fields appear.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create encrypted dataset with valid passphrase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open Create File System dialog.
-2. Select parent, enter name 'test_pass_enc'.
-3. Toggle Encryption ON.
-4. Enter matching passphrases (8+ characters).
-5. Click Create.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dataset is created successfully. Notification: 'File System Created'. Dataset appears in list with a lock icon.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reject passphrase under 8 characters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open Create File System dialog.
-2. Enable Encryption.
-3. Enter passphrase 'short' (5 chars).
-4. Enter same in Confirm field.
-5. Click Create.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Validation error displayed: passphrase requires at least 8 characters. Dataset is NOT created.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reject mismatched passphrases</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open Create File System dialog.
-2. Enable Encryption.
-3. Enter 'Password123!' in Passphrase.
-4. Enter 'Different123!' in Confirm.
-5. Click Create.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Validation error: passphrases do not match. Dataset is NOT created.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reject empty passphrase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open Create File System dialog.
-2. Enable Encryption.
-3. Leave passphrase fields empty.
-4. Click Create.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Validation error displayed. Dataset is NOT created.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eye icon toggles passphrase visibility</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open Create File System dialog.
-2. Enable Encryption.
-3. Enter a passphrase.
-4. Click the eye icon next to the passphrase field.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Passphrase text toggles between masked and visible (plaintext). Icon changes between eye/eye-slash.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Encryption toggle off hides encryption fields</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open Create File System dialog.
-2. Toggle Encryption ON.
-3. Toggle Encryption OFF.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Passphrase fields and Key Source selector (if visible) disappear.</t>
   </si>
   <si>
     <t xml:space="preserve">Create FS - KMS Encryption</t>
@@ -463,20 +352,6 @@
   </si>
   <si>
     <t xml:space="preserve">Dataset is created. Notification confirms success. Dataset appears in list with lock icon. Running 'zfs get keylocation test_kms_enc' shows 'file://' path.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reject KMS creation with no policy selected</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open Create FS → enable encryption → select KMS.
-2. Leave policy dropdown at 'Select a key policy...'.
-3. Click Create.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Validation error: a policy must be selected. Dataset is NOT created.</t>
   </si>
   <si>
     <t xml:space="preserve">4.7</t>
@@ -495,123 +370,6 @@
     <t xml:space="preserve">UI switches cleanly between modes. Passphrase fields show/hide. Policy dropdown shows/hides. Previously selected policy is retained when switching back.</t>
   </si>
   <si>
-    <t xml:space="preserve">4.8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Empty policy dropdown when no policies exist</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Remove all key policies from the Storage Encryption module.
-2. Open Create FS → enable encryption → select KMS.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Policy dropdown shows 'Select a key policy...' but has no options to select. User cannot proceed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unlock - Passphrase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Context menu shows 'Unlock File System' for locked dataset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Have a passphrase-encrypted dataset that is locked and unmounted.
-2. Navigate to Datasets tab.
-3. Click the three-dot menu on the locked dataset.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Context menu includes 'Unlock File System' with green highlight on hover.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unlock with correct passphrase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click 'Unlock File System' on a locked passphrase dataset.
-2. Enter the correct passphrase.
-3. Leave 'Mount File System' toggled ON.
-4. Click 'Unlock'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dataset unlocks and mounts. Notification: 'Dataset Unlocked'. Lock icon changes to open. 'Mounted' column shows 'yes'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unlock with incorrect passphrase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click 'Unlock File System' on a locked passphrase dataset.
-2. Enter a wrong passphrase.
-3. Click 'Unlock'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Error message displayed below passphrase field. Dataset remains locked.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unlock without mounting</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click 'Unlock File System' on a locked passphrase dataset.
-2. Enter correct passphrase.
-3. Toggle 'Mount File System' OFF.
-4. Click 'Unlock'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dataset unlocks (key loaded). Lock icon changes to open. 'Mounted' column remains 'no'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unlock with Force Mount option</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click 'Unlock File System' on a locked passphrase dataset.
-2. Enter correct passphrase.
-3. Toggle 'Mount File System' ON.
-4. Toggle 'Forcefully Mount File System' ON.
-5. Click 'Unlock'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dataset unlocks and mounts (with -f flag). Notification confirms success.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cancel unlock dialog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click 'Unlock File System' on a locked dataset.
-2. Click 'Cancel'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dialog closes. Dataset remains locked.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eye icon toggles passphrase visibility in unlock dialog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click 'Unlock File System' on a locked passphrase dataset.
-2. Enter a passphrase.
-3. Click the eye icon.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Passphrase toggles between masked and visible text.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Unlock - KMS</t>
   </si>
   <si>
@@ -707,6 +465,9 @@
 2. Click 'Cancel'.</t>
   </si>
   <si>
+    <t xml:space="preserve">Dialog closes. Dataset remains locked.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lock &amp; Unmount</t>
   </si>
   <si>
@@ -797,117 +558,6 @@
   </si>
   <si>
     <t xml:space="preserve">Dataset mounts. 'Mounted' column changes to 'yes'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Change Passphrase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Change Passphrase menu item for passphrase-encrypted dataset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Have a passphrase-encrypted (non-KMS) dataset that is unlocked.
-2. Click context menu.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menu includes 'Change Passphrase'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Change Passphrase hidden for KMS-managed dataset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Have a KMS-managed encrypted dataset that is unlocked.
-2. Click context menu.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menu does NOT include 'Change Passphrase'. (KMS keys are managed externally.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Successfully change passphrase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click 'Change Passphrase'.
-2. Enter new passphrase (8+ chars) in 'New Passphrase'.
-3. Enter same in 'Confirm New Passphrase'.
-4. Click 'Change'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Success notification: passphrase changed. Important reminder about noting passphrase is visible. Dialog closes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reject mismatched new passphrases</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click 'Change Passphrase'.
-2. Enter 'NewPass123!' in New.
-3. Enter 'Different123!' in Confirm.
-4. Click 'Change'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Validation error: passphrases do not match. Passphrase is NOT changed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reject short new passphrase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click 'Change Passphrase'.
-2. Enter 'short' in both fields.
-3. Click 'Change'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Validation error: minimum 8 characters. Passphrase is NOT changed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Important passphrase reminder is visible</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click 'Change Passphrase'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Red text visible: 'Important: Please note your passphrase carefully. If it is lost, it cannot be retrieved or reset.'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cancel change passphrase dialog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click 'Change Passphrase'.
-2. Click 'Cancel'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dialog closes. Passphrase is NOT changed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Change Passphrase hidden for locked dataset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Have a passphrase-encrypted dataset that is locked.
-2. Check context menu.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menu does NOT include 'Change Passphrase'. Only 'Unlock File System' is shown for encryption operations.</t>
   </si>
   <si>
     <t xml:space="preserve">Context Menu - KMS Items</t>
@@ -1163,22 +813,6 @@
     <t xml:space="preserve">Error: dataset already exists. Second dataset is NOT created.</t>
   </si>
   <si>
-    <t xml:space="preserve">Create Zvol</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create Zvol button opens dialog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Navigate to Datasets tab.
-2. Click 'Create Zvol'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zvol creation dialog opens.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Navigation &amp; Refresh</t>
   </si>
   <si>
@@ -1234,19 +868,6 @@
   </si>
   <si>
     <t xml:space="preserve">Security &amp; Edge Cases</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Passphrase not logged or persisted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Create an encrypted dataset with a passphrase.
-2. Check browser dev tools console and network tab.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Passphrase is not visible in console logs, network requests (except the cockpit spawn call), or localStorage.</t>
   </si>
   <si>
     <t xml:space="preserve">15.2</t>
@@ -1263,19 +884,6 @@
     <t xml:space="preserve">The actual encryption key (DEK) is never shown in the UI, console, or network responses visible to the browser.</t>
   </si>
   <si>
-    <t xml:space="preserve">15.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Concurrent lock/unlock operations</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open two browser tabs.
-2. Try to unlock the same locked dataset simultaneously.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One operation succeeds; the other shows an error or the dataset is already unlocked. No data corruption.</t>
-  </si>
-  <si>
     <t xml:space="preserve">15.4</t>
   </si>
   <si>
@@ -1300,20 +908,6 @@
   </si>
   <si>
     <t xml:space="preserve">UI toggles cleanly without errors. Final state is correctly reflected (fields show/hide consistently).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Passphrase with special characters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Create encrypted dataset with passphrase containing special chars: P@$$w0rd!&lt;&gt;"&amp;
-2. Lock the dataset.
-3. Unlock with the same passphrase.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dataset creates and unlocks successfully with special characters in the passphrase.</t>
   </si>
   <si>
     <t xml:space="preserve">15.7</t>
@@ -1328,161 +922,6 @@
   </si>
   <si>
     <t xml:space="preserve">Name is rejected as invalid (special characters). No script execution. No XSS vulnerability.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pool Creation Wizard - Encryption</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Encryption available in Pool Creation Wizard file system step</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Start Pool Creation Wizard.
-2. Proceed to the File System configuration step.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Encryption toggle and passphrase/KMS fields are available, same as standalone Create File System.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Review tab shows encryption settings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Configure encryption in the Pool Creation Wizard.
-2. Proceed to Review tab.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Review tab displays the encryption settings: enabled/disabled, key source (passphrase or KMS), and policy name if KMS.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notifications</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Success notification on dataset creation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Create any dataset successfully.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Green success notification appears briefly with 'File System Created' or similar message.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Success notification on lock/unlock</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Lock or unlock a dataset successfully.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Success notification: 'Dataset Locked' or 'Dataset Unlocked' (or 'Successfully unlocked via KMS').</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Error notification on failed operation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Attempt an operation that fails (e.g., wrong passphrase).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Red error notification with descriptive error message.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Success notification on passphrase change</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Successfully change a passphrase.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Success notification confirming passphrase was changed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mount/unmount notifications</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Mount or unmount a dataset.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Success notification: 'File System Mounted' or 'File System Unmounted'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Loading &amp; Error States</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Loading spinner during unlock operation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click Unlock on a dataset. Enter passphrase. Click Unlock.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A spinner appears on the Unlock button. Button text changes to 'Unlocking...'. Button is disabled during operation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Loading spinner during lock operation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click Lock on a dataset. Confirm.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spinner appears on the Lock button. Text changes to 'Locking...'. Button is disabled.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Loading spinner during passphrase change</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter valid passphrases in Change Passphrase. Click Change.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spinner on Change button. Text: 'Changing...'. Button disabled until operation completes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dataset list loading spinner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Navigate to Datasets tab while data is loading.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A loading spinner is shown in the table area until datasets are fully loaded.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Control plane loading state in dashboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open Dashboard while control plane data is loading.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Encryption Governance card shows a loading spinner until posture data is fetched.</t>
   </si>
   <si>
     <t xml:space="preserve">How to Use This Test Plan</t>
@@ -2054,7 +1493,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J101"/>
+  <dimension ref="A1:J63"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
@@ -2386,7 +1825,7 @@
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
     </row>
-    <row r="15" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
         <v>81</v>
       </c>
@@ -2408,7 +1847,7 @@
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
     </row>
-    <row r="16" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
         <v>81</v>
       </c>
@@ -2430,7 +1869,7 @@
       <c r="I16" s="5"/>
       <c r="J16" s="5"/>
     </row>
-    <row r="17" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
         <v>81</v>
       </c>
@@ -2452,7 +1891,7 @@
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
     </row>
-    <row r="18" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
         <v>81</v>
       </c>
@@ -2496,7 +1935,7 @@
       <c r="I19" s="5"/>
       <c r="J19" s="5"/>
     </row>
-    <row r="20" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
         <v>81</v>
       </c>
@@ -2518,53 +1957,53 @@
       <c r="I20" s="5"/>
       <c r="J20" s="5"/>
     </row>
-    <row r="21" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="B21" s="5" t="s">
+    <row r="21" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5" t="s">
+      <c r="B21" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="C21" s="4"/>
+      <c r="D21" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="F21" s="5" t="s">
+      <c r="E21" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-    </row>
-    <row r="22" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="F21" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
+    </row>
+    <row r="22" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B22" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4" t="s">
+      <c r="C22" s="5"/>
+      <c r="D22" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>115</v>
@@ -2584,9 +2023,9 @@
       <c r="I23" s="5"/>
       <c r="J23" s="5"/>
     </row>
-    <row r="24" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>119</v>
@@ -2606,9 +2045,9 @@
       <c r="I24" s="5"/>
       <c r="J24" s="5"/>
     </row>
-    <row r="25" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>123</v>
@@ -2628,9 +2067,9 @@
       <c r="I25" s="5"/>
       <c r="J25" s="5"/>
     </row>
-    <row r="26" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>127</v>
@@ -2650,9 +2089,9 @@
       <c r="I26" s="5"/>
       <c r="J26" s="5"/>
     </row>
-    <row r="27" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>131</v>
@@ -2672,75 +2111,75 @@
       <c r="I27" s="5"/>
       <c r="J27" s="5"/>
     </row>
-    <row r="28" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="B28" s="5" t="s">
+    <row r="28" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="C28" s="5"/>
-      <c r="D28" s="5" t="s">
+      <c r="B28" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="E28" s="5" t="s">
+      <c r="C28" s="4"/>
+      <c r="D28" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="F28" s="5" t="s">
+      <c r="E28" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="G28" s="5"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="5"/>
-      <c r="J28" s="5"/>
-    </row>
-    <row r="29" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F28" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="4"/>
+      <c r="J28" s="4"/>
+    </row>
+    <row r="29" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>110</v>
+        <v>135</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C29" s="5"/>
       <c r="D29" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G29" s="5"/>
       <c r="H29" s="5"/>
       <c r="I29" s="5"/>
       <c r="J29" s="5"/>
     </row>
-    <row r="30" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="B30" s="4" t="s">
+    <row r="30" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B30" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4" t="s">
+      <c r="C30" s="5"/>
+      <c r="D30" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="F30" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="G30" s="4"/>
-      <c r="H30" s="4"/>
-      <c r="I30" s="4"/>
-      <c r="J30" s="4"/>
-    </row>
-    <row r="31" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G30" s="5"/>
+      <c r="H30" s="5"/>
+      <c r="I30" s="5"/>
+      <c r="J30" s="5"/>
+    </row>
+    <row r="31" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>148</v>
@@ -2760,9 +2199,9 @@
       <c r="I31" s="5"/>
       <c r="J31" s="5"/>
     </row>
-    <row r="32" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>152</v>
@@ -2782,9 +2221,9 @@
       <c r="I32" s="5"/>
       <c r="J32" s="5"/>
     </row>
-    <row r="33" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>156</v>
@@ -2804,9 +2243,9 @@
       <c r="I33" s="5"/>
       <c r="J33" s="5"/>
     </row>
-    <row r="34" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>160</v>
@@ -2827,74 +2266,74 @@
       <c r="J34" s="5"/>
     </row>
     <row r="35" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="B35" s="5" t="s">
+      <c r="A35" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="C35" s="5"/>
-      <c r="D35" s="5" t="s">
+      <c r="B35" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="E35" s="5" t="s">
+      <c r="C35" s="4"/>
+      <c r="D35" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="F35" s="5" t="s">
+      <c r="E35" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="G35" s="5"/>
-      <c r="H35" s="5"/>
-      <c r="I35" s="5"/>
-      <c r="J35" s="5"/>
+      <c r="F35" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="G35" s="4"/>
+      <c r="H35" s="4"/>
+      <c r="I35" s="4"/>
+      <c r="J35" s="4"/>
     </row>
     <row r="36" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>143</v>
+        <v>164</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G36" s="5"/>
       <c r="H36" s="5"/>
       <c r="I36" s="5"/>
       <c r="J36" s="5"/>
     </row>
-    <row r="37" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="B37" s="4" t="s">
+    <row r="37" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="B37" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4" t="s">
+      <c r="C37" s="5"/>
+      <c r="D37" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="E37" s="4" t="s">
+      <c r="E37" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="F37" s="4" t="s">
+      <c r="F37" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="G37" s="4"/>
-      <c r="H37" s="4"/>
-      <c r="I37" s="4"/>
-      <c r="J37" s="4"/>
-    </row>
-    <row r="38" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G37" s="5"/>
+      <c r="H37" s="5"/>
+      <c r="I37" s="5"/>
+      <c r="J37" s="5"/>
+    </row>
+    <row r="38" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>177</v>
@@ -2916,7 +2355,7 @@
     </row>
     <row r="39" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>181</v>
@@ -2936,242 +2375,242 @@
       <c r="I39" s="5"/>
       <c r="J39" s="5"/>
     </row>
-    <row r="40" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="B40" s="5" t="s">
+    <row r="40" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="C40" s="5"/>
-      <c r="D40" s="5" t="s">
+      <c r="B40" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="E40" s="5" t="s">
+      <c r="C40" s="4"/>
+      <c r="D40" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="F40" s="5" t="s">
+      <c r="E40" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="G40" s="5"/>
-      <c r="H40" s="5"/>
-      <c r="I40" s="5"/>
-      <c r="J40" s="5"/>
+      <c r="F40" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="G40" s="4"/>
+      <c r="H40" s="4"/>
+      <c r="I40" s="4"/>
+      <c r="J40" s="4"/>
     </row>
     <row r="41" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G41" s="5"/>
       <c r="H41" s="5"/>
       <c r="I41" s="5"/>
       <c r="J41" s="5"/>
     </row>
-    <row r="42" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="B42" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="C42" s="5"/>
-      <c r="D42" s="5" t="s">
+    <row r="42" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="E42" s="5" t="s">
+      <c r="B42" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="F42" s="5" t="s">
+      <c r="C42" s="4"/>
+      <c r="D42" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="G42" s="5"/>
-      <c r="H42" s="5"/>
-      <c r="I42" s="5"/>
-      <c r="J42" s="5"/>
+      <c r="E42" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="G42" s="4"/>
+      <c r="H42" s="4"/>
+      <c r="I42" s="4"/>
+      <c r="J42" s="4"/>
     </row>
     <row r="43" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>172</v>
+        <v>194</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C43" s="5"/>
       <c r="D43" s="5" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>167</v>
+        <v>202</v>
       </c>
       <c r="G43" s="5"/>
       <c r="H43" s="5"/>
       <c r="I43" s="5"/>
       <c r="J43" s="5"/>
     </row>
-    <row r="44" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="C44" s="4"/>
-      <c r="D44" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="E44" s="4" t="s">
+    <row r="44" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="B44" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="F44" s="4" t="s">
+      <c r="C44" s="5"/>
+      <c r="D44" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="G44" s="4"/>
-      <c r="H44" s="4"/>
-      <c r="I44" s="4"/>
-      <c r="J44" s="4"/>
-    </row>
-    <row r="45" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E44" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="G44" s="5"/>
+      <c r="H44" s="5"/>
+      <c r="I44" s="5"/>
+      <c r="J44" s="5"/>
+    </row>
+    <row r="45" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="5" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G45" s="5"/>
       <c r="H45" s="5"/>
       <c r="I45" s="5"/>
       <c r="J45" s="5"/>
     </row>
-    <row r="46" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C46" s="5"/>
       <c r="D46" s="5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G46" s="5"/>
       <c r="H46" s="5"/>
       <c r="I46" s="5"/>
       <c r="J46" s="5"/>
     </row>
-    <row r="47" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C47" s="5"/>
       <c r="D47" s="5" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G47" s="5"/>
       <c r="H47" s="5"/>
       <c r="I47" s="5"/>
       <c r="J47" s="5"/>
     </row>
-    <row r="48" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C48" s="5"/>
       <c r="D48" s="5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G48" s="5"/>
       <c r="H48" s="5"/>
       <c r="I48" s="5"/>
       <c r="J48" s="5"/>
     </row>
-    <row r="49" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="B49" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="C49" s="5"/>
-      <c r="D49" s="5" t="s">
+    <row r="49" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="E49" s="5" t="s">
+      <c r="B49" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="F49" s="5" t="s">
+      <c r="C49" s="4"/>
+      <c r="D49" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="G49" s="5"/>
-      <c r="H49" s="5"/>
-      <c r="I49" s="5"/>
-      <c r="J49" s="5"/>
-    </row>
-    <row r="50" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E49" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="G49" s="4"/>
+      <c r="H49" s="4"/>
+      <c r="I49" s="4"/>
+      <c r="J49" s="4"/>
+    </row>
+    <row r="50" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>200</v>
+        <v>222</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C50" s="5"/>
       <c r="D50" s="5" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="G50" s="5"/>
       <c r="H50" s="5"/>
@@ -3179,109 +2618,109 @@
       <c r="J50" s="5"/>
     </row>
     <row r="51" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="C51" s="4"/>
-      <c r="D51" s="4" t="s">
+      <c r="A51" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="B51" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="E51" s="4" t="s">
+      <c r="C51" s="5"/>
+      <c r="D51" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="F51" s="4" t="s">
+      <c r="E51" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="G51" s="4"/>
-      <c r="H51" s="4"/>
-      <c r="I51" s="4"/>
-      <c r="J51" s="4"/>
-    </row>
-    <row r="52" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F51" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="G51" s="5"/>
+      <c r="H51" s="5"/>
+      <c r="I51" s="5"/>
+      <c r="J51" s="5"/>
+    </row>
+    <row r="52" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C52" s="5"/>
       <c r="D52" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F52" s="5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G52" s="5"/>
       <c r="H52" s="5"/>
       <c r="I52" s="5"/>
       <c r="J52" s="5"/>
     </row>
-    <row r="53" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C53" s="5"/>
       <c r="D53" s="5" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="G53" s="5"/>
       <c r="H53" s="5"/>
       <c r="I53" s="5"/>
       <c r="J53" s="5"/>
     </row>
-    <row r="54" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="B54" s="5" t="s">
-        <v>242</v>
-      </c>
-      <c r="C54" s="5"/>
-      <c r="D54" s="5" t="s">
+    <row r="54" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="E54" s="5" t="s">
+      <c r="B54" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="F54" s="5" t="s">
+      <c r="C54" s="4"/>
+      <c r="D54" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="G54" s="5"/>
-      <c r="H54" s="5"/>
-      <c r="I54" s="5"/>
-      <c r="J54" s="5"/>
-    </row>
-    <row r="55" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E54" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="G54" s="4"/>
+      <c r="H54" s="4"/>
+      <c r="I54" s="4"/>
+      <c r="J54" s="4"/>
+    </row>
+    <row r="55" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>229</v>
+        <v>243</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C55" s="5"/>
       <c r="D55" s="5" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="F55" s="5" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="G55" s="5"/>
       <c r="H55" s="5"/>
@@ -3290,20 +2729,20 @@
     </row>
     <row r="56" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>229</v>
+        <v>243</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C56" s="5"/>
       <c r="D56" s="5" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="F56" s="5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="G56" s="5"/>
       <c r="H56" s="5"/>
@@ -3312,20 +2751,20 @@
     </row>
     <row r="57" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
-        <v>229</v>
+        <v>243</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C57" s="5"/>
       <c r="D57" s="5" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="F57" s="5" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="G57" s="5"/>
       <c r="H57" s="5"/>
@@ -3333,87 +2772,69 @@
       <c r="J57" s="5"/>
     </row>
     <row r="58" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="B58" s="5" t="s">
-        <v>258</v>
-      </c>
-      <c r="C58" s="5"/>
-      <c r="D58" s="5" t="s">
-        <v>259</v>
-      </c>
-      <c r="E58" s="5" t="s">
+      <c r="A58" s="4" t="s">
         <v>260</v>
       </c>
-      <c r="F58" s="5" t="s">
+      <c r="B58" s="4"/>
+      <c r="C58" s="4"/>
+      <c r="D58" s="4"/>
+      <c r="E58" s="4"/>
+      <c r="F58" s="4"/>
+      <c r="G58" s="4"/>
+      <c r="H58" s="4"/>
+      <c r="I58" s="4"/>
+      <c r="J58" s="4"/>
+    </row>
+    <row r="59" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="B59" s="5" t="s">
         <v>261</v>
       </c>
-      <c r="G58" s="5"/>
-      <c r="H58" s="5"/>
-      <c r="I58" s="5"/>
-      <c r="J58" s="5"/>
-    </row>
-    <row r="59" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="4" t="s">
+      <c r="C59" s="5"/>
+      <c r="D59" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="B59" s="4" t="s">
+      <c r="E59" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="C59" s="4"/>
-      <c r="D59" s="4" t="s">
+      <c r="F59" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="E59" s="4" t="s">
-        <v>265</v>
-      </c>
-      <c r="F59" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="G59" s="4"/>
-      <c r="H59" s="4"/>
-      <c r="I59" s="4"/>
-      <c r="J59" s="4"/>
-    </row>
-    <row r="60" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="5" t="s">
-        <v>262</v>
-      </c>
-      <c r="B60" s="5" t="s">
-        <v>267</v>
-      </c>
+      <c r="G59" s="5"/>
+      <c r="H59" s="5"/>
+      <c r="I59" s="5"/>
+      <c r="J59" s="5"/>
+    </row>
+    <row r="60" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="5"/>
+      <c r="B60" s="5"/>
       <c r="C60" s="5"/>
-      <c r="D60" s="5" t="s">
-        <v>268</v>
-      </c>
-      <c r="E60" s="5" t="s">
-        <v>269</v>
-      </c>
-      <c r="F60" s="5" t="s">
-        <v>270</v>
-      </c>
+      <c r="D60" s="5"/>
+      <c r="E60" s="5"/>
+      <c r="F60" s="5"/>
       <c r="G60" s="5"/>
       <c r="H60" s="5"/>
       <c r="I60" s="5"/>
       <c r="J60" s="5"/>
     </row>
-    <row r="61" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="C61" s="5"/>
       <c r="D61" s="5" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="F61" s="5" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="G61" s="5"/>
       <c r="H61" s="5"/>
@@ -3422,20 +2843,20 @@
     </row>
     <row r="62" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="C62" s="5"/>
       <c r="D62" s="5" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="F62" s="5" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="G62" s="5"/>
       <c r="H62" s="5"/>
@@ -3444,861 +2865,25 @@
     </row>
     <row r="63" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="C63" s="5"/>
       <c r="D63" s="5" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F63" s="5" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="G63" s="5"/>
       <c r="H63" s="5"/>
       <c r="I63" s="5"/>
       <c r="J63" s="5"/>
-    </row>
-    <row r="64" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="B64" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="C64" s="4"/>
-      <c r="D64" s="4" t="s">
-        <v>285</v>
-      </c>
-      <c r="E64" s="4" t="s">
-        <v>286</v>
-      </c>
-      <c r="F64" s="4" t="s">
-        <v>287</v>
-      </c>
-      <c r="G64" s="4"/>
-      <c r="H64" s="4"/>
-      <c r="I64" s="4"/>
-      <c r="J64" s="4"/>
-    </row>
-    <row r="65" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="5" t="s">
-        <v>283</v>
-      </c>
-      <c r="B65" s="5" t="s">
-        <v>288</v>
-      </c>
-      <c r="C65" s="5"/>
-      <c r="D65" s="5" t="s">
-        <v>289</v>
-      </c>
-      <c r="E65" s="5" t="s">
-        <v>290</v>
-      </c>
-      <c r="F65" s="5" t="s">
-        <v>291</v>
-      </c>
-      <c r="G65" s="5"/>
-      <c r="H65" s="5"/>
-      <c r="I65" s="5"/>
-      <c r="J65" s="5"/>
-    </row>
-    <row r="66" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="4" t="s">
-        <v>292</v>
-      </c>
-      <c r="B66" s="4" t="s">
-        <v>293</v>
-      </c>
-      <c r="C66" s="4"/>
-      <c r="D66" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="E66" s="4" t="s">
-        <v>295</v>
-      </c>
-      <c r="F66" s="4" t="s">
-        <v>296</v>
-      </c>
-      <c r="G66" s="4"/>
-      <c r="H66" s="4"/>
-      <c r="I66" s="4"/>
-      <c r="J66" s="4"/>
-    </row>
-    <row r="67" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="B67" s="5" t="s">
-        <v>297</v>
-      </c>
-      <c r="C67" s="5"/>
-      <c r="D67" s="5" t="s">
-        <v>298</v>
-      </c>
-      <c r="E67" s="5" t="s">
-        <v>299</v>
-      </c>
-      <c r="F67" s="5" t="s">
-        <v>300</v>
-      </c>
-      <c r="G67" s="5"/>
-      <c r="H67" s="5"/>
-      <c r="I67" s="5"/>
-      <c r="J67" s="5"/>
-    </row>
-    <row r="68" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="B68" s="5" t="s">
-        <v>301</v>
-      </c>
-      <c r="C68" s="5"/>
-      <c r="D68" s="5" t="s">
-        <v>302</v>
-      </c>
-      <c r="E68" s="5" t="s">
-        <v>303</v>
-      </c>
-      <c r="F68" s="5" t="s">
-        <v>304</v>
-      </c>
-      <c r="G68" s="5"/>
-      <c r="H68" s="5"/>
-      <c r="I68" s="5"/>
-      <c r="J68" s="5"/>
-    </row>
-    <row r="69" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="B69" s="5" t="s">
-        <v>305</v>
-      </c>
-      <c r="C69" s="5"/>
-      <c r="D69" s="5" t="s">
-        <v>306</v>
-      </c>
-      <c r="E69" s="5" t="s">
-        <v>295</v>
-      </c>
-      <c r="F69" s="5" t="s">
-        <v>307</v>
-      </c>
-      <c r="G69" s="5"/>
-      <c r="H69" s="5"/>
-      <c r="I69" s="5"/>
-      <c r="J69" s="5"/>
-    </row>
-    <row r="70" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="B70" s="5" t="s">
-        <v>308</v>
-      </c>
-      <c r="C70" s="5"/>
-      <c r="D70" s="5" t="s">
-        <v>309</v>
-      </c>
-      <c r="E70" s="5" t="s">
-        <v>310</v>
-      </c>
-      <c r="F70" s="5" t="s">
-        <v>311</v>
-      </c>
-      <c r="G70" s="5"/>
-      <c r="H70" s="5"/>
-      <c r="I70" s="5"/>
-      <c r="J70" s="5"/>
-    </row>
-    <row r="71" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="B71" s="5" t="s">
-        <v>312</v>
-      </c>
-      <c r="C71" s="5"/>
-      <c r="D71" s="5" t="s">
-        <v>313</v>
-      </c>
-      <c r="E71" s="5" t="s">
-        <v>314</v>
-      </c>
-      <c r="F71" s="5" t="s">
-        <v>315</v>
-      </c>
-      <c r="G71" s="5"/>
-      <c r="H71" s="5"/>
-      <c r="I71" s="5"/>
-      <c r="J71" s="5"/>
-    </row>
-    <row r="72" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="B72" s="5" t="s">
-        <v>316</v>
-      </c>
-      <c r="C72" s="5"/>
-      <c r="D72" s="5" t="s">
-        <v>317</v>
-      </c>
-      <c r="E72" s="5" t="s">
-        <v>318</v>
-      </c>
-      <c r="F72" s="5" t="s">
-        <v>319</v>
-      </c>
-      <c r="G72" s="5"/>
-      <c r="H72" s="5"/>
-      <c r="I72" s="5"/>
-      <c r="J72" s="5"/>
-    </row>
-    <row r="73" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="4" t="s">
-        <v>320</v>
-      </c>
-      <c r="B73" s="4" t="s">
-        <v>321</v>
-      </c>
-      <c r="C73" s="4"/>
-      <c r="D73" s="4" t="s">
-        <v>322</v>
-      </c>
-      <c r="E73" s="4" t="s">
-        <v>323</v>
-      </c>
-      <c r="F73" s="4" t="s">
-        <v>324</v>
-      </c>
-      <c r="G73" s="4"/>
-      <c r="H73" s="4"/>
-      <c r="I73" s="4"/>
-      <c r="J73" s="4"/>
-    </row>
-    <row r="74" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="5" t="s">
-        <v>320</v>
-      </c>
-      <c r="B74" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="C74" s="5"/>
-      <c r="D74" s="5" t="s">
-        <v>326</v>
-      </c>
-      <c r="E74" s="5" t="s">
-        <v>327</v>
-      </c>
-      <c r="F74" s="5" t="s">
-        <v>328</v>
-      </c>
-      <c r="G74" s="5"/>
-      <c r="H74" s="5"/>
-      <c r="I74" s="5"/>
-      <c r="J74" s="5"/>
-    </row>
-    <row r="75" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="5" t="s">
-        <v>320</v>
-      </c>
-      <c r="B75" s="5" t="s">
-        <v>329</v>
-      </c>
-      <c r="C75" s="5"/>
-      <c r="D75" s="5" t="s">
-        <v>330</v>
-      </c>
-      <c r="E75" s="5" t="s">
-        <v>331</v>
-      </c>
-      <c r="F75" s="5" t="s">
-        <v>332</v>
-      </c>
-      <c r="G75" s="5"/>
-      <c r="H75" s="5"/>
-      <c r="I75" s="5"/>
-      <c r="J75" s="5"/>
-    </row>
-    <row r="76" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="5" t="s">
-        <v>320</v>
-      </c>
-      <c r="B76" s="5" t="s">
-        <v>333</v>
-      </c>
-      <c r="C76" s="5"/>
-      <c r="D76" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="E76" s="5" t="s">
-        <v>335</v>
-      </c>
-      <c r="F76" s="5" t="s">
-        <v>336</v>
-      </c>
-      <c r="G76" s="5"/>
-      <c r="H76" s="5"/>
-      <c r="I76" s="5"/>
-      <c r="J76" s="5"/>
-    </row>
-    <row r="77" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="5" t="s">
-        <v>320</v>
-      </c>
-      <c r="B77" s="5" t="s">
-        <v>337</v>
-      </c>
-      <c r="C77" s="5"/>
-      <c r="D77" s="5" t="s">
-        <v>338</v>
-      </c>
-      <c r="E77" s="5" t="s">
-        <v>339</v>
-      </c>
-      <c r="F77" s="5" t="s">
-        <v>340</v>
-      </c>
-      <c r="G77" s="5"/>
-      <c r="H77" s="5"/>
-      <c r="I77" s="5"/>
-      <c r="J77" s="5"/>
-    </row>
-    <row r="78" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="4" t="s">
-        <v>341</v>
-      </c>
-      <c r="B78" s="4" t="s">
-        <v>342</v>
-      </c>
-      <c r="C78" s="4"/>
-      <c r="D78" s="4" t="s">
-        <v>343</v>
-      </c>
-      <c r="E78" s="4" t="s">
-        <v>344</v>
-      </c>
-      <c r="F78" s="4" t="s">
-        <v>345</v>
-      </c>
-      <c r="G78" s="4"/>
-      <c r="H78" s="4"/>
-      <c r="I78" s="4"/>
-      <c r="J78" s="4"/>
-    </row>
-    <row r="79" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="4" t="s">
-        <v>346</v>
-      </c>
-      <c r="B79" s="4" t="s">
-        <v>347</v>
-      </c>
-      <c r="C79" s="4"/>
-      <c r="D79" s="4" t="s">
-        <v>348</v>
-      </c>
-      <c r="E79" s="4" t="s">
-        <v>349</v>
-      </c>
-      <c r="F79" s="4" t="s">
-        <v>350</v>
-      </c>
-      <c r="G79" s="4"/>
-      <c r="H79" s="4"/>
-      <c r="I79" s="4"/>
-      <c r="J79" s="4"/>
-    </row>
-    <row r="80" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="B80" s="5" t="s">
-        <v>351</v>
-      </c>
-      <c r="C80" s="5"/>
-      <c r="D80" s="5" t="s">
-        <v>352</v>
-      </c>
-      <c r="E80" s="5" t="s">
-        <v>353</v>
-      </c>
-      <c r="F80" s="5" t="s">
-        <v>354</v>
-      </c>
-      <c r="G80" s="5"/>
-      <c r="H80" s="5"/>
-      <c r="I80" s="5"/>
-      <c r="J80" s="5"/>
-    </row>
-    <row r="81" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="B81" s="5" t="s">
-        <v>355</v>
-      </c>
-      <c r="C81" s="5"/>
-      <c r="D81" s="5" t="s">
-        <v>356</v>
-      </c>
-      <c r="E81" s="5" t="s">
-        <v>357</v>
-      </c>
-      <c r="F81" s="5" t="s">
-        <v>358</v>
-      </c>
-      <c r="G81" s="5"/>
-      <c r="H81" s="5"/>
-      <c r="I81" s="5"/>
-      <c r="J81" s="5"/>
-    </row>
-    <row r="82" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="B82" s="5" t="s">
-        <v>359</v>
-      </c>
-      <c r="C82" s="5"/>
-      <c r="D82" s="5" t="s">
-        <v>360</v>
-      </c>
-      <c r="E82" s="5" t="s">
-        <v>361</v>
-      </c>
-      <c r="F82" s="5" t="s">
-        <v>362</v>
-      </c>
-      <c r="G82" s="5"/>
-      <c r="H82" s="5"/>
-      <c r="I82" s="5"/>
-      <c r="J82" s="5"/>
-    </row>
-    <row r="83" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="4" t="s">
-        <v>363</v>
-      </c>
-      <c r="B83" s="4" t="s">
-        <v>364</v>
-      </c>
-      <c r="C83" s="4"/>
-      <c r="D83" s="4" t="s">
-        <v>365</v>
-      </c>
-      <c r="E83" s="4" t="s">
-        <v>366</v>
-      </c>
-      <c r="F83" s="4" t="s">
-        <v>367</v>
-      </c>
-      <c r="G83" s="4"/>
-      <c r="H83" s="4"/>
-      <c r="I83" s="4"/>
-      <c r="J83" s="4"/>
-    </row>
-    <row r="84" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="5" t="s">
-        <v>363</v>
-      </c>
-      <c r="B84" s="5" t="s">
-        <v>368</v>
-      </c>
-      <c r="C84" s="5"/>
-      <c r="D84" s="5" t="s">
-        <v>369</v>
-      </c>
-      <c r="E84" s="5" t="s">
-        <v>370</v>
-      </c>
-      <c r="F84" s="5" t="s">
-        <v>371</v>
-      </c>
-      <c r="G84" s="5"/>
-      <c r="H84" s="5"/>
-      <c r="I84" s="5"/>
-      <c r="J84" s="5"/>
-    </row>
-    <row r="85" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="5" t="s">
-        <v>363</v>
-      </c>
-      <c r="B85" s="5" t="s">
-        <v>372</v>
-      </c>
-      <c r="C85" s="5"/>
-      <c r="D85" s="5" t="s">
-        <v>373</v>
-      </c>
-      <c r="E85" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="F85" s="5" t="s">
-        <v>375</v>
-      </c>
-      <c r="G85" s="5"/>
-      <c r="H85" s="5"/>
-      <c r="I85" s="5"/>
-      <c r="J85" s="5"/>
-    </row>
-    <row r="86" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="5" t="s">
-        <v>363</v>
-      </c>
-      <c r="B86" s="5" t="s">
-        <v>376</v>
-      </c>
-      <c r="C86" s="5"/>
-      <c r="D86" s="5" t="s">
-        <v>377</v>
-      </c>
-      <c r="E86" s="5" t="s">
-        <v>378</v>
-      </c>
-      <c r="F86" s="5" t="s">
-        <v>379</v>
-      </c>
-      <c r="G86" s="5"/>
-      <c r="H86" s="5"/>
-      <c r="I86" s="5"/>
-      <c r="J86" s="5"/>
-    </row>
-    <row r="87" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="5" t="s">
-        <v>363</v>
-      </c>
-      <c r="B87" s="5" t="s">
-        <v>380</v>
-      </c>
-      <c r="C87" s="5"/>
-      <c r="D87" s="5" t="s">
-        <v>381</v>
-      </c>
-      <c r="E87" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="F87" s="5" t="s">
-        <v>383</v>
-      </c>
-      <c r="G87" s="5"/>
-      <c r="H87" s="5"/>
-      <c r="I87" s="5"/>
-      <c r="J87" s="5"/>
-    </row>
-    <row r="88" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="5" t="s">
-        <v>363</v>
-      </c>
-      <c r="B88" s="5" t="s">
-        <v>384</v>
-      </c>
-      <c r="C88" s="5"/>
-      <c r="D88" s="5" t="s">
-        <v>385</v>
-      </c>
-      <c r="E88" s="5" t="s">
-        <v>386</v>
-      </c>
-      <c r="F88" s="5" t="s">
-        <v>387</v>
-      </c>
-      <c r="G88" s="5"/>
-      <c r="H88" s="5"/>
-      <c r="I88" s="5"/>
-      <c r="J88" s="5"/>
-    </row>
-    <row r="89" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="5" t="s">
-        <v>363</v>
-      </c>
-      <c r="B89" s="5" t="s">
-        <v>388</v>
-      </c>
-      <c r="C89" s="5"/>
-      <c r="D89" s="5" t="s">
-        <v>389</v>
-      </c>
-      <c r="E89" s="5" t="s">
-        <v>390</v>
-      </c>
-      <c r="F89" s="5" t="s">
-        <v>391</v>
-      </c>
-      <c r="G89" s="5"/>
-      <c r="H89" s="5"/>
-      <c r="I89" s="5"/>
-      <c r="J89" s="5"/>
-    </row>
-    <row r="90" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="B90" s="4" t="s">
-        <v>393</v>
-      </c>
-      <c r="C90" s="4"/>
-      <c r="D90" s="4" t="s">
-        <v>394</v>
-      </c>
-      <c r="E90" s="4" t="s">
-        <v>395</v>
-      </c>
-      <c r="F90" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="G90" s="4"/>
-      <c r="H90" s="4"/>
-      <c r="I90" s="4"/>
-      <c r="J90" s="4"/>
-    </row>
-    <row r="91" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="5" t="s">
-        <v>392</v>
-      </c>
-      <c r="B91" s="5" t="s">
-        <v>397</v>
-      </c>
-      <c r="C91" s="5"/>
-      <c r="D91" s="5" t="s">
-        <v>398</v>
-      </c>
-      <c r="E91" s="5" t="s">
-        <v>399</v>
-      </c>
-      <c r="F91" s="5" t="s">
-        <v>400</v>
-      </c>
-      <c r="G91" s="5"/>
-      <c r="H91" s="5"/>
-      <c r="I91" s="5"/>
-      <c r="J91" s="5"/>
-    </row>
-    <row r="92" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="4" t="s">
-        <v>401</v>
-      </c>
-      <c r="B92" s="4" t="s">
-        <v>402</v>
-      </c>
-      <c r="C92" s="4"/>
-      <c r="D92" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="E92" s="4" t="s">
-        <v>404</v>
-      </c>
-      <c r="F92" s="4" t="s">
-        <v>405</v>
-      </c>
-      <c r="G92" s="4"/>
-      <c r="H92" s="4"/>
-      <c r="I92" s="4"/>
-      <c r="J92" s="4"/>
-    </row>
-    <row r="93" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="5" t="s">
-        <v>401</v>
-      </c>
-      <c r="B93" s="5" t="s">
-        <v>406</v>
-      </c>
-      <c r="C93" s="5"/>
-      <c r="D93" s="5" t="s">
-        <v>407</v>
-      </c>
-      <c r="E93" s="5" t="s">
-        <v>408</v>
-      </c>
-      <c r="F93" s="5" t="s">
-        <v>409</v>
-      </c>
-      <c r="G93" s="5"/>
-      <c r="H93" s="5"/>
-      <c r="I93" s="5"/>
-      <c r="J93" s="5"/>
-    </row>
-    <row r="94" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="5" t="s">
-        <v>401</v>
-      </c>
-      <c r="B94" s="5" t="s">
-        <v>410</v>
-      </c>
-      <c r="C94" s="5"/>
-      <c r="D94" s="5" t="s">
-        <v>411</v>
-      </c>
-      <c r="E94" s="5" t="s">
-        <v>412</v>
-      </c>
-      <c r="F94" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="G94" s="5"/>
-      <c r="H94" s="5"/>
-      <c r="I94" s="5"/>
-      <c r="J94" s="5"/>
-    </row>
-    <row r="95" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="5" t="s">
-        <v>401</v>
-      </c>
-      <c r="B95" s="5" t="s">
-        <v>414</v>
-      </c>
-      <c r="C95" s="5"/>
-      <c r="D95" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="E95" s="5" t="s">
-        <v>416</v>
-      </c>
-      <c r="F95" s="5" t="s">
-        <v>417</v>
-      </c>
-      <c r="G95" s="5"/>
-      <c r="H95" s="5"/>
-      <c r="I95" s="5"/>
-      <c r="J95" s="5"/>
-    </row>
-    <row r="96" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="5" t="s">
-        <v>401</v>
-      </c>
-      <c r="B96" s="5" t="s">
-        <v>418</v>
-      </c>
-      <c r="C96" s="5"/>
-      <c r="D96" s="5" t="s">
-        <v>419</v>
-      </c>
-      <c r="E96" s="5" t="s">
-        <v>420</v>
-      </c>
-      <c r="F96" s="5" t="s">
-        <v>421</v>
-      </c>
-      <c r="G96" s="5"/>
-      <c r="H96" s="5"/>
-      <c r="I96" s="5"/>
-      <c r="J96" s="5"/>
-    </row>
-    <row r="97" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="4" t="s">
-        <v>422</v>
-      </c>
-      <c r="B97" s="4" t="s">
-        <v>423</v>
-      </c>
-      <c r="C97" s="4"/>
-      <c r="D97" s="4" t="s">
-        <v>424</v>
-      </c>
-      <c r="E97" s="4" t="s">
-        <v>425</v>
-      </c>
-      <c r="F97" s="4" t="s">
-        <v>426</v>
-      </c>
-      <c r="G97" s="4"/>
-      <c r="H97" s="4"/>
-      <c r="I97" s="4"/>
-      <c r="J97" s="4"/>
-    </row>
-    <row r="98" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="B98" s="5" t="s">
-        <v>427</v>
-      </c>
-      <c r="C98" s="5"/>
-      <c r="D98" s="5" t="s">
-        <v>428</v>
-      </c>
-      <c r="E98" s="5" t="s">
-        <v>429</v>
-      </c>
-      <c r="F98" s="5" t="s">
-        <v>430</v>
-      </c>
-      <c r="G98" s="5"/>
-      <c r="H98" s="5"/>
-      <c r="I98" s="5"/>
-      <c r="J98" s="5"/>
-    </row>
-    <row r="99" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="B99" s="5" t="s">
-        <v>431</v>
-      </c>
-      <c r="C99" s="5"/>
-      <c r="D99" s="5" t="s">
-        <v>432</v>
-      </c>
-      <c r="E99" s="5" t="s">
-        <v>433</v>
-      </c>
-      <c r="F99" s="5" t="s">
-        <v>434</v>
-      </c>
-      <c r="G99" s="5"/>
-      <c r="H99" s="5"/>
-      <c r="I99" s="5"/>
-      <c r="J99" s="5"/>
-    </row>
-    <row r="100" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="B100" s="5" t="s">
-        <v>435</v>
-      </c>
-      <c r="C100" s="5"/>
-      <c r="D100" s="5" t="s">
-        <v>436</v>
-      </c>
-      <c r="E100" s="5" t="s">
-        <v>437</v>
-      </c>
-      <c r="F100" s="5" t="s">
-        <v>438</v>
-      </c>
-      <c r="G100" s="5"/>
-      <c r="H100" s="5"/>
-      <c r="I100" s="5"/>
-      <c r="J100" s="5"/>
-    </row>
-    <row r="101" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="B101" s="5" t="s">
-        <v>439</v>
-      </c>
-      <c r="C101" s="5"/>
-      <c r="D101" s="5" t="s">
-        <v>440</v>
-      </c>
-      <c r="E101" s="5" t="s">
-        <v>441</v>
-      </c>
-      <c r="F101" s="5" t="s">
-        <v>442</v>
-      </c>
-      <c r="G101" s="5"/>
-      <c r="H101" s="5"/>
-      <c r="I101" s="5"/>
-      <c r="J101" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -4324,122 +2909,122 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>443</v>
+        <v>277</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>444</v>
+        <v>278</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>445</v>
+        <v>279</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>446</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>447</v>
+        <v>281</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>448</v>
+        <v>282</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>449</v>
+        <v>283</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>450</v>
+        <v>284</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>451</v>
+        <v>285</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>452</v>
+        <v>286</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>453</v>
+        <v>287</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>454</v>
+        <v>288</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>455</v>
+        <v>289</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>456</v>
+        <v>290</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>457</v>
+        <v>291</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>458</v>
+        <v>292</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>459</v>
+        <v>293</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>460</v>
+        <v>294</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>461</v>
+        <v>295</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>462</v>
+        <v>296</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>463</v>
+        <v>297</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>464</v>
+        <v>298</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>465</v>
+        <v>299</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>466</v>
+        <v>300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>